<commit_message>
feat: Update error comparison Excel file for summary replication
</commit_message>
<xml_diff>
--- a/main/summary_replication/error_comparison.xlsx
+++ b/main/summary_replication/error_comparison.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orincon\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\ReScience-PINNs\main\summary_replication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14E7039A-999B-4444-9D62-DEDDC63BF5D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACF8008-0C63-4EF7-89BE-BD2D78F87C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
   <si>
     <t>Model / Parameter</t>
   </si>
@@ -76,31 +76,18 @@
   </si>
   <si>
     <t>relative L₂ error</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Continuous forward — Burgers equation </t>
-  </si>
-  <si>
-    <t>Continuous inverse — Burgers equations  (% error)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discrete forward — Burgers equation  </t>
-  </si>
-  <si>
-    <t>Discrete inverse — Burgers equation  (% error)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.000E+00"/>
+  <numFmts count="3">
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000\%"/>
     <numFmt numFmtId="167" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -143,6 +130,19 @@
       <b/>
       <sz val="10"/>
       <color rgb="FF993C1D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -213,51 +213,55 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -535,301 +539,293 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="14">
+      <c r="B3" s="9">
         <v>1.97E-3</v>
       </c>
-      <c r="C3" s="15">
+      <c r="C3" s="14">
         <v>1.307E-3</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="4">
         <f>(C3-B3)/ABS(B3)</f>
         <v>-0.33654822335025381</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
     </row>
     <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="8">
         <v>7.7999999999999999E-4</v>
       </c>
-      <c r="C5" s="5">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="C5" s="15">
+        <v>6.9999999999999994E-5</v>
+      </c>
+      <c r="D5" s="4">
         <f>(C5-B5)/ABS(B5)</f>
-        <v>7.9743589743589745</v>
+        <v>-0.91025641025641024</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="5">
         <v>4.67</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="16">
         <v>1.8640000000000001</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <f>(C6-B6)/ABS(B6)</f>
         <v>-0.60085653104925052</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="5">
         <v>0.17</v>
       </c>
-      <c r="C7" s="5">
-        <v>2.9000000000000001E-2</v>
-      </c>
-      <c r="D7" s="6">
+      <c r="C7" s="15">
+        <v>2.9E-4</v>
+      </c>
+      <c r="D7" s="4">
         <f>(C7-B7)/ABS(B7)</f>
-        <v>-0.8294117647058824</v>
+        <v>-0.99829411764705878</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="5">
         <v>5.7</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="16">
         <v>3.29</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <f>(C8-B8)/ABS(B8)</f>
         <v>-0.42280701754385969</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="9">
         <v>6.9899999999999997E-3</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="14">
         <v>1.307E-3</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <f>(C10-B10)/ABS(B10)</f>
         <v>-0.81301859799713871</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="8">
         <v>2.3000000000000001E-4</v>
       </c>
-      <c r="C12" s="5">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="D12" s="6">
+      <c r="C12" s="8">
+        <v>4.0000000000000003E-5</v>
+      </c>
+      <c r="D12" s="4">
         <f>(C12-B12)/ABS(B12)</f>
-        <v>16.391304347826086</v>
+        <v>-0.82608695652173914</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="8">
         <v>6.0000000000000002E-5</v>
       </c>
-      <c r="C13" s="5">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="D13" s="6">
+      <c r="C13" s="8">
+        <v>5.0000000000000002E-5</v>
+      </c>
+      <c r="D13" s="4">
         <f>(C13-B13)/ABS(B13)</f>
-        <v>82.333333333333329</v>
+        <v>-0.16666666666666666</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="8">
         <v>5.6999999999999998E-4</v>
       </c>
-      <c r="C14" s="9">
-        <v>0.11899999999999999</v>
-      </c>
-      <c r="D14" s="10">
+      <c r="C14" s="8">
+        <v>1.1900000000000001E-3</v>
+      </c>
+      <c r="D14" s="6">
         <f>(C14-B14)/ABS(B14)</f>
-        <v>207.7719298245614</v>
+        <v>1.0877192982456143</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="8">
         <v>1.7000000000000001E-4</v>
       </c>
-      <c r="C15" s="11">
-        <v>4.8000000000000001E-2</v>
-      </c>
-      <c r="D15" s="10">
+      <c r="C15" s="17">
+        <v>4.8000000000000001E-4</v>
+      </c>
+      <c r="D15" s="6">
         <f>(C15-B15)/ABS(B15)</f>
-        <v>281.35294117647055</v>
+        <v>1.8235294117647058</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17">
-        <v>6.7000000000000002E-4</v>
-      </c>
+      <c r="A17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>5</v>
-      </c>
+      <c r="A19" s="11"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A20" s="11"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>7</v>
-      </c>
+      <c r="A21" s="11"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="A22" s="11"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24">
-        <v>8.1999999999999998E-4</v>
-      </c>
+      <c r="A24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>5</v>
-      </c>
+      <c r="A26" s="11"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A27" s="11"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
-        <v>7</v>
-      </c>
+      <c r="A28" s="11"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="A29" s="11"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A25:D25"/>
+  <mergeCells count="4">
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>